<commit_message>
All changes for 2026 - so far
</commit_message>
<xml_diff>
--- a/AMAS Standards List.xlsx
+++ b/AMAS Standards List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lrosenth/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lrosenth/amas-tech-reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BFF054E-7F71-AC42-8545-0E40BF1E98B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834A08E8-64E2-6A49-9D67-039761065730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="45660" yWindow="5120" windowWidth="28040" windowHeight="21880" xr2:uid="{98DD96FF-909E-BB43-A3CF-B6AA999C76C6}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="116">
   <si>
     <t>Category</t>
   </si>
@@ -375,6 +375,9 @@
   </si>
   <si>
     <t>ISO 21617-3</t>
+  </si>
+  <si>
+    <t>Content Credentials (C2PA)</t>
   </si>
 </sst>
 </file>
@@ -828,7 +831,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>7</v>
+        <v>115</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>8</v>
@@ -1328,6 +1331,24 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Meeting_x0020_Date xmlns="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1" xsi:nil="true"/>
+    <Source xmlns="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BC603E13C3A73340A6732121C1853D0C" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a9cb6de74c33d4e3470966593f12d6e0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1" xmlns:ns3="2828a09b-4f48-432d-9559-a1f724b08bae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c2d1b904aad086a408849faa6bfb2a80" ns2:_="" ns3:_="">
     <xsd:import namespace="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1"/>
@@ -1486,25 +1507,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Meeting_x0020_Date xmlns="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1" xsi:nil="true"/>
-    <Source xmlns="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF031DC2-3F49-456B-8ACE-BC811F5E6293}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24240BB2-E93E-416C-84FF-0227B25E9DCD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAAAC215-9937-4C7B-B4BD-7F77D1E34F91}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1521,22 +1542,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24240BB2-E93E-416C-84FF-0227B25E9DCD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="43f3aac0-5e6c-4529-8eca-b318fd6f3bb1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF031DC2-3F49-456B-8ACE-BC811F5E6293}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>